<commit_message>
feat: enhance menu dialog and image controls for narrow screens
chore: update Supabase CLI to version 2.122.0

feat: create private schema and tables for restaurant production storage and transactions

feat: implement cron jobs for session cleanup and log retention

fix: update audit snapshot function to include audit records

fix: modify auto_accept function to include audit row keys

test: add unit tests for cloud store and currency functionalities

test: implement tests for staff authentication and management

chore: add Vercel configuration for deployment
</commit_message>
<xml_diff>
--- a/public/templates/template-menu-restoOS.xlsx
+++ b/public/templates/template-menu-restoOS.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menu" sheetId="1" r:id="R6c5a0c0265024b4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="Rc6c2ba81b2494fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menu" sheetId="1" r:id="R47bd58a061a444b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="Rff9889fdf8fd43d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -296,7 +296,7 @@
         <x:v>Kategori</x:v>
       </x:c>
       <x:c r="C1" s="2" t="str">
-        <x:v>Harga (IDR)</x:v>
+        <x:v>Harga</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
         <x:v>Deskripsi</x:v>
@@ -3446,15 +3446,15 @@
         <x:v>Kategori</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Wajib, 1–40 karakter. Contoh: Hidangan utama.</x:v>
+        <x:v>Wajib, 1–40 karakter. Gunakan kategori restoran Anda.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" t="str">
-        <x:v>Harga (IDR)</x:v>
+        <x:v>Harga</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Angka bulat positif. Ketik 30000, bukan Rp30.000. Harga final.</x:v>
+        <x:v>Angka bulat positif dalam mata uang dasar, tanpa simbol atau pemisah ribuan.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
@@ -3486,52 +3486,30 @@
         <x:v>Foto menu</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Belum didukung. Upload foto menyusul setelah Supabase Storage terhubung.</x:v>
+        <x:v>Foto diunggah melalui formulir menu; impor Excel mempertahankan foto yang ada.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1"/>
     <x:row r="14" ht="25" customHeight="1">
-      <x:c r="A14" t="str">
-        <x:v>Contoh saja: isi data Anda pada sheet Menu</x:v>
-      </x:c>
-      <x:c r="B14" t="str"/>
-      <x:c r="C14" t="str"/>
-      <x:c r="D14" t="str"/>
-      <x:c r="E14" t="str"/>
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="2" t="str">
-        <x:v>Nama menu</x:v>
-      </x:c>
-      <x:c r="B15" s="2" t="str">
-        <x:v>Kategori</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
-        <x:v>Harga (IDR)</x:v>
-      </x:c>
-      <x:c r="D15" s="2" t="str">
-        <x:v>Deskripsi</x:v>
-      </x:c>
-      <x:c r="E15" s="2" t="str">
-        <x:v>Tersedia</x:v>
-      </x:c>
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>Nasi goreng</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>Hidangan utama</x:v>
-      </x:c>
-      <x:c r="C16" s="6" t="n">
-        <x:v>30000</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>Nasi goreng dengan telur.</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>Ya</x:v>
-      </x:c>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>